<commit_message>
test(rf-006,rf-007): close SHAP explainer and doctor review test gaps
Adds unit tests for shap_explainer.py (RF-006) and integration tests
for the AI analysis review flow (RF-007), then updates the Plan de
Pruebas (v1.2) and Catalogo de Pruebas to reflect both as Implementado.
Adds Acta_Reunion_3 documenting the work.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
+++ b/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
@@ -1231,7 +1231,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Automática (por implementar)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -1241,12 +1241,12 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>Sin evidencia de prueba dedicada al módulo</t>
-        </is>
-      </c>
-      <c r="N12" s="6" t="inlineStr">
-        <is>
-          <t>En progreso (50%)</t>
+          <t>14/14 casos superados: load_model, explain_prediction (factores positivos/negativos, orden por importancia, top-3 predicciones, valores SHAP crudos), explain_batch, get_feature_importance_summary</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>GAP: shap_explainer.py no cuenta con test dedicado; solo existe test_patient_friendly_explainer.py (capa de presentación)</t>
+          <t>GAP cerrado: se agregó test_shap_explainer.py, que prueba el módulo núcleo shap_explainer.py de forma aislada del stub global usado por otras suites (mock de joblib.load y shap.TreeExplainer)</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Automática (por implementar)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Sin test de servicio/integración dedicado (solo test de modelo AIAnalysis)</t>
-        </is>
-      </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>No iniciado (0%)</t>
+          <t>13/13 casos unitarios (100% statements/functions/lines) + 11/11 casos de integración end-to-end sobre /api/v1/ai-analysis</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>GAP: existe AIAnalysis.test.ts (modelo) pero no test de aiAnalysisReviewService.ts ni de aiAnalysisReviewRoutes.ts</t>
+          <t>GAP cerrado: se agregaron aiAnalysisReviewService.test.ts (unitario) y aiAnalysisReview.integration.test.ts (integración con mongodb-memory-server), cubriendo aprobar/rechazar/ajustar, firma electrónica, autorización por rol y bloqueo de doble revisión</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(e2e): close functional test catalog gaps for RF-005/006/007/011/012
Add end-to-end flow tests covering clinical coherence validation,
SHAP explanation delivery to doctors, doctor panel review with
electronic signature, educational content personalization, and
health center geolocation search. Closes CP-005-F, CP-006-F,
CP-007-F, CP-011-F and CP-012-F in the test catalog.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
+++ b/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
@@ -3085,12 +3085,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>POST /api/v1/symptom-analyzer/ml-analyze con síntomas coherentes retorna is_clinically_coherent=true y coherence_warnings vacío; el análisis queda disponible en GET /api/v1/ai-analysis/pending para revisión médica.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>POST /api/v1/symptom-analyzer/ml-analyze con síntomas graves y urgencia clasificada como baja retorna is_clinically_coherent=false junto con coherence_warnings explícitos; la predicción no se descarta automáticamente sino que queda en la cola de revisión y el médico la rechaza tras evaluarla (POST /api/v1/ai-analysis/:id/review con decision=rejected).</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
@@ -3135,22 +3135,22 @@
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe un flujo de sistema dedicado; la validación se ejerce como parte del mismo flujo funcional de RF-002 (Análisis de Síntomas con IA).</t>
+          <t>flows.test.ts &gt; 'Flujo Completo: Validación de Coherencia Médica ante Síntomas Contradictorios (RF-005)' - 1/1 test. Verifica que el sistema expone la incoherencia clínica sin ocultarla y que el flujo exige revisión médica antes de descartar la predicción.</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>Cubierto indirectamente por flows.test.ts (Flujo Completo: Análisis de Síntomas con IA); se recomienda un caso de flujo explícito con síntomas incoherentes</t>
+          <t>Cierra el GAP de CP-005-F. Depende de CP-002 y del passthrough is_clinically_coherent/coherence_warnings ya existente en aiIntegration.ts (RF-005).</t>
         </is>
       </c>
     </row>
@@ -3620,12 +3620,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>POST /api/v1/symptom-analyzer/ml-analyze con síntomas respiratorios retorna 200 con disease + explanation (positive_factors/negative_factors/decision_factors SHAP); el análisis se persiste y el médico lo consulta vía GET /api/v1/ai-analysis/:id antes de aprobarlo con firma electrónica.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>N/A a nivel de sistema - cubierto por CP-006-I (fallback a Random Forest y error 500 cuando ambos modelos fallan al cargar).</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr">
@@ -3670,22 +3670,22 @@
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe un flujo de sistema dedicado que valide la entrega de la explicación SHAP al usuario final.</t>
+          <t>flows.test.ts &gt; 'Flujo Completo: Explicabilidad SHAP y Panel del Doctor (RF-006, RF-007)' - 1/1 test. Verifica que el médico recibe la explicación SHAP junto con el diagnóstico y puede revisarla antes de firmar la aprobación.</t>
         </is>
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="U33" s="2" t="inlineStr">
         <is>
-          <t>Depende de que se resuelva primero el GAP de integración (endpoint de explicación)</t>
+          <t>Cierra el GAP de CP-006-F, una vez resuelto el GAP de integración previo (CP-006-I). Comparte flujo de sistema con CP-007-F.</t>
         </is>
       </c>
     </row>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>El médico consulta GET /api/v1/ai-analysis/pending, revisa el detalle en GET /api/v1/ai-analysis/:id y aprueba la predicción con firma electrónica vía POST /api/v1/ai-analysis/:id/review (decision=approved); el estado persistido pasa a 'approved'.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>El médico rechaza una predicción marcada como clínicamente incoherente por el sistema (decision=rejected), cubierto en el mismo flujo que CP-005-F; CP-007-I cubre además casos de error a nivel de endpoint (firma faltante, doble revisión, acceso denegado a paciente).</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
@@ -4205,22 +4205,22 @@
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe un flujo de sistema (flows.test.ts) dedicado al panel del doctor; el ciclo completo ya se valida end-to-end a nivel de integración (11/11 casos).</t>
+          <t>flows.test.ts &gt; 'Flujo Completo: Explicabilidad SHAP y Panel del Doctor (RF-006, RF-007)' - 1/1 test (ciclo completo: cola de pendientes -&gt; detalle -&gt; revisión con firma electrónica).</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="U38" s="2" t="inlineStr">
         <is>
-          <t>Cubierto en profundidad por aiAnalysisReview.integration.test.ts; se recomienda añadir un flujo explícito en flows.test.ts</t>
+          <t>Cierra el GAP de CP-007-F, complementando la cobertura de endpoint ya existente en aiAnalysisReview.integration.test.ts (CP-007-I).</t>
         </is>
       </c>
     </row>
@@ -6295,12 +6295,12 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Un paciente diagnosticado con 'asma' consulta GET /api/v1/educational-content y recibe contenido específico de asma y contenido general, sin recibir contenido de otras condiciones (EPOC); al consultar el detalle se incrementa el viewCount.</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>N/A a nivel de sistema - cubierto por CP-011-I (401 sin autenticación, 404 contenido inexistente, 403 gestión por rol no autorizado, 400 categoría inválida).</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr">
@@ -6345,22 +6345,22 @@
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe un flujo de sistema dedicado en flows.test.ts para el módulo educativo.</t>
+          <t>flows.test.ts &gt; 'Flujo Completo: Personalización de Contenido Educativo tras Diagnóstico (RF-011)' - 1/1 test.</t>
         </is>
       </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="U58" s="2" t="inlineStr">
         <is>
-          <t>Depende de resolver primero el GAP de integración</t>
+          <t>Cierra el GAP de CP-011-F, una vez resuelto el GAP de integración previo (CP-011-I) y el bug de colisión de claves $or en EducationalContentModel.findRelevantFor.</t>
         </is>
       </c>
     </row>
@@ -6830,12 +6830,12 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Un paciente registrado busca GET /api/v1/health-centers/nearby con su ubicación actual y respiratoryOnly=true; recibe el centro de salud con atención respiratoria más cercano, ordenado por distanceKm.</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>N/A a nivel de sistema - cubierto por healthCenters.integration.test.ts (401 sin autenticación, 400 coordenadas faltantes).</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -6860,7 +6860,7 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
@@ -6880,22 +6880,22 @@
       </c>
       <c r="R63" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe un flujo de sistema/E2E dedicado a la búsqueda de centros de salud desde la perspectiva del usuario final.</t>
+          <t>flows.test.ts &gt; 'Flujo Completo: Búsqueda Geoespacial de Centros de Salud (RF-012)' - 1/1 test.</t>
         </is>
       </c>
       <c r="S63" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="U63" s="2" t="inlineStr">
         <is>
-          <t>Recomendación: agregar un flujo en flows.test.ts o un spec Cypress móvil dedicado</t>
+          <t>Cierra el GAP de CP-012-F (registro -&gt; búsqueda geoespacial), complementando healthCenters.integration.test.ts (CP-012-I).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(performance): close performance test catalog gaps for RF-003/005/006/007/011/012
Adds dedicated performance/benchmark coverage for the 6 remaining
CP-XXX-R gaps: cough audio spectral analysis latency, ml-analyze
coherence-validation SLA, SHAP explain_prediction() overhead
benchmark, and doctor review/educational-content/health-centers
endpoint SLAs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
+++ b/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
@@ -2122,12 +2122,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Con librosa reconfigurado (vía monkeypatch sobre el stub global de conftest.py) para devolver arreglos numpy con la forma real de un audio de tos de ~2s a 22050Hz, CoughAnalysisService._extract_audio_features() y analyze() completan la extracción espectral (zcr, centroide, rolloff, bandwidth, mfcc, chroma, rms) y la clasificación de características de tos dentro de los umbrales definidos (p50&lt;200ms, p95&lt;500ms, p99&lt;1000ms).</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Si la extracción de features o la clasificación de características exceden los umbrales de latencia definidos, las aserciones p50/p95/p99 fallan y el test reporta el incumplimiento del SLA.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -2172,22 +2172,22 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe una prueba de rendimiento dedicada al pipeline de audio; solo se mide performance del ensemble de síntomas y de clasificación de imágenes genérica.</t>
+          <t>Implementado en ai-services/tests/performance/test_prediction_latency.py::TestCoughAudioSpectralAnalysisLatency (test_audio_feature_extraction_latency_distribution, test_full_cough_analysis_pipeline_latency). Se reconfiguró el stub global de librosa para devolver arreglos numpy con la forma real de un audio de ~2s, midiendo el costo real de las reducciones (np.mean/std/max) y de la lógica de clasificación de CoughAnalysisService sin requerir la instalación real de librosa.</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>Recomendación: extender ai-services/tests/performance/test_prediction_latency.py con un caso específico de audio/espectrograma</t>
+          <t>Complementa CP-003-I/CP-003-F ya cerrados; evidencia que el pipeline de audio cumple el SLA de lectura estándar (P50/P95/P99 definidos en el propio archivo).</t>
         </is>
       </c>
     </row>
@@ -3192,12 +3192,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>POST /api/v1/symptom-analyzer/ml-analyze (con aiIntegrationService.analyzeSymptomsML mockeado devolviendo is_clinically_coherent/coherence_warnings) responde dentro del SLA de escritura (mean&lt;350ms, p95&lt;600ms, p99&lt;900ms), confirmando que el passthrough de los campos de coherencia médica no añade overhead relevante al endpoint.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Si el endpoint excede el SLA de escritura definido, la aserción assertSLA(...) falla indicando el incumplimiento.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
@@ -3242,22 +3242,22 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe una prueba de rendimiento dedicada; el impacto se mide de forma agregada dentro del SLA general de RF-002 (CP-002, &lt;3 s).</t>
+          <t>Implementado en backend/tests/performance/api-performance.perf.test.ts, describe 'Performance — ML Symptom Analyzer (coherencia médica) Endpoint'. Se agregó evidencia directa y dedicada al endpoint /ml-analyze, en reemplazo de la cobertura transversal previamente documentada (CP-002).</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>Cubierto de forma transversal por CP-002 (Prueba de rendimiento) y api-performance.perf.test.ts</t>
+          <t>Sustituye la cobertura transversal previamente documentada (CP-002) por una prueba de rendimiento dedicada al endpoint /ml-analyze.</t>
         </is>
       </c>
     </row>
@@ -3727,12 +3727,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>El benchmark test_shap_explanation_overhead_benchmark (pytest-benchmark) mide explain_prediction() de SHAPDiseaseExplainer usando un modelo/vectorizer simulados y lo compara contra una predicción cruda (model.predict + predict_proba) llamada directamente, documentando el overhead real que añade el cálculo y post-procesamiento de valores SHAP.</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Si explain_prediction() lanza una excepción o no retorna 'shap_values'/'disease' como se espera, la aserción del test falla.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
@@ -3777,22 +3777,22 @@
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe una prueba de rendimiento dedicada al cálculo de SHAP.</t>
+          <t>Implementado en ai-services/tests/performance/test_benchmark.py::TestSHAPExplanationOverheadBenchmark. Carga el módulo real shap_explainer.py (bypaseando el stub global de conftest.py) y compara mediante el patrón A/B ya usado en test_with_vs_without_personalization_benchmark (baseline llamado directamente, solo la ruta con SHAP se pasa a benchmark()).</t>
         </is>
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr">
         <is>
-          <t>Recomendación: incluir benchmark de explain_prediction() en ai-services/tests/performance/test_benchmark.py</t>
+          <t>Complementa CP-006-F (explicabilidad funcional) con evidencia de su costo en tiempo.</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4262,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>GET /api/v1/ai-analysis/pending y POST /api/v1/ai-analysis/:id/review responden dentro de sus SLA de lectura/escritura (read: mean&lt;200/p95&lt;400/p99&lt;600ms; write: mean&lt;350/p95&lt;600/p99&lt;900ms).</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Si alguno de los dos endpoints excede su SLA, assertSLA(...) falla e identifica el endpoint incumplido.</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
@@ -4312,22 +4312,22 @@
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe una prueba de rendimiento dedicada a los endpoints de /api/v1/ai-analysis.</t>
+          <t>Implementado en backend/tests/performance/api-performance.perf.test.ts, describe 'Performance — AI Analysis Review Endpoints' (GET /ai-analysis/pending sobre datos sembrados; POST /ai-analysis/:id/review con un análisis nuevo por iteración, dado que cada análisis solo admite una revisión).</t>
         </is>
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>Recomendación: extender api-performance.perf.test.ts con SLA para GET /ai-analysis/pending y POST /ai-analysis/:id/review</t>
+          <t>Complementa CP-007-F/CP-007-I ya cerrados con evidencia de tiempos de respuesta.</t>
         </is>
       </c>
     </row>
@@ -6402,12 +6402,12 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>GET /api/v1/educational-content responde dentro del SLA de lectura (mean&lt;200ms, p95&lt;400ms, p99&lt;600ms), incluyendo la lógica de personalización por historial clínico.</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Si el endpoint excede el SLA de lectura definido, assertSLA(...) falla.</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O59" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr">
@@ -6452,22 +6452,22 @@
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe una prueba de rendimiento dedicada al módulo educativo.</t>
+          <t>Implementado en backend/tests/performance/api-performance.perf.test.ts, describe 'Performance — Educational Content Endpoint'.</t>
         </is>
       </c>
       <c r="S59" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="U59" s="2" t="inlineStr">
         <is>
-          <t>Recomendación: extender api-performance.perf.test.ts con SLA para el endpoint de contenido educativo</t>
+          <t>Complementa CP-011-F/CP-011-I ya cerrados.</t>
         </is>
       </c>
     </row>
@@ -6937,12 +6937,12 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>GET /api/v1/health-centers/nearby responde dentro del SLA de búsqueda (mean&lt;250ms, p95&lt;450ms, p99&lt;700ms).</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>N/A — caso marcado como Pendiente (ver Observaciones); no existe evidencia real de test para derivar un escenario.</t>
+          <t>Si la búsqueda geoespacial excede el SLA definido, assertSLA(...) falla.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>GAP: sin prueba dedicada a este nivel</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Automática (pendiente)</t>
+          <t>Automática</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -6987,22 +6987,22 @@
       </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>GAP: no existe una prueba de rendimiento dedicada a este endpoint.</t>
+          <t>Implementado en backend/tests/performance/api-performance.perf.test.ts, describe 'Performance — Health Centers Nearby Endpoint'.</t>
         </is>
       </c>
       <c r="S64" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="U64" s="2" t="inlineStr">
         <is>
-          <t>Recomendación: extender api-performance.perf.test.ts con SLA para el endpoint de centros de salud</t>
+          <t>Complementa CP-012-F/CP-012-I ya cerrados.</t>
         </is>
       </c>
     </row>

</xml_diff>